<commit_message>
Update human behaviour in AddictO_Human_behaviour_Defs.xlsx
</commit_message>
<xml_diff>
--- a/inputs/AddictO_Human_behaviour_Defs.xlsx
+++ b/inputs/AddictO_Human_behaviour_Defs.xlsx
@@ -644,7 +644,7 @@
           <t>point prevalence tobacco smoking abstinence</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n"/>
       <c r="F3" s="3" t="n"/>
       <c r="G3" s="3" t="inlineStr">
         <is>
@@ -1852,7 +1852,7 @@
           <t>abstinence from a behaviour</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="n"/>
       <c r="F22" s="3" t="n"/>
       <c r="G22" s="3" t="inlineStr">
         <is>
@@ -5078,7 +5078,7 @@
           <t>continuous abstinence</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr"/>
+      <c r="C78" s="2" t="n"/>
       <c r="D78" s="2" t="n"/>
       <c r="E78" s="2" t="n"/>
       <c r="F78" s="2" t="n"/>
@@ -10129,56 +10129,67 @@
       <c r="U172" s="3" t="n"/>
     </row>
     <row r="173">
-      <c r="A173" t="inlineStr">
+      <c r="A173" s="5" t="inlineStr">
         <is>
           <t>BCIO:042000</t>
         </is>
       </c>
-      <c r="B173" t="inlineStr">
+      <c r="B173" s="5" t="inlineStr">
         <is>
           <t>human behaviour</t>
         </is>
       </c>
-      <c r="C173" t="inlineStr">
+      <c r="C173" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Individual human behaviour or population behaviour. </t>
         </is>
       </c>
-      <c r="D173" t="inlineStr">
+      <c r="D173" s="5" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="G173" t="inlineStr">
-        <is>
-          <t>Human behaviour</t>
-        </is>
-      </c>
-      <c r="L173" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="Q173" t="inlineStr">
+      <c r="E173" s="5" t="n"/>
+      <c r="F173" s="5" t="n"/>
+      <c r="G173" s="5" t="inlineStr">
+        <is>
+          <t>Human behaviour</t>
+        </is>
+      </c>
+      <c r="H173" s="5" t="n"/>
+      <c r="I173" s="5" t="n"/>
+      <c r="J173" s="5" t="n"/>
+      <c r="K173" s="5" t="n"/>
+      <c r="L173" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M173" s="5" t="n"/>
+      <c r="N173" s="5" t="n"/>
+      <c r="O173" s="5" t="n"/>
+      <c r="P173" s="5" t="n"/>
+      <c r="Q173" s="5" t="inlineStr">
         <is>
           <t>JH</t>
         </is>
       </c>
-      <c r="R173" t="inlineStr">
+      <c r="R173" s="5" t="inlineStr">
         <is>
           <t>Process</t>
         </is>
       </c>
-      <c r="S173" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="T173" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="S173" s="5" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="T173" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U173" s="5" t="n"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -14628,7 +14639,7 @@
           <t>data item</t>
         </is>
       </c>
-      <c r="E265" s="3" t="inlineStr"/>
+      <c r="E265" s="3" t="n"/>
       <c r="F265" s="3" t="n"/>
       <c r="G265" s="3" t="inlineStr">
         <is>
@@ -14890,7 +14901,7 @@
           <t>tobacco smoking abstinence</t>
         </is>
       </c>
-      <c r="E270" s="3" t="inlineStr"/>
+      <c r="E270" s="3" t="n"/>
       <c r="F270" s="3" t="inlineStr">
         <is>
           <t>The period of time over which the person is abstinent needs to be specified. Is is usually 7 days.</t>
@@ -19483,7 +19494,7 @@
           <t>successful continuous abstinence</t>
         </is>
       </c>
-      <c r="C365" s="2" t="inlineStr"/>
+      <c r="C365" s="2" t="n"/>
       <c r="D365" s="2" t="n"/>
       <c r="E365" s="2" t="n"/>
       <c r="F365" s="2" t="n"/>
@@ -19664,7 +19675,7 @@
         </is>
       </c>
       <c r="C369" s="2" t="n"/>
-      <c r="D369" s="2" t="inlineStr"/>
+      <c r="D369" s="2" t="n"/>
       <c r="E369" s="2" t="n"/>
       <c r="F369" s="2" t="n"/>
       <c r="G369" s="2" t="inlineStr">
@@ -20329,8 +20340,8 @@
           <t>abstinence from a behaviour</t>
         </is>
       </c>
-      <c r="E383" s="3" t="inlineStr"/>
-      <c r="F383" s="3" t="inlineStr"/>
+      <c r="E383" s="3" t="n"/>
+      <c r="F383" s="3" t="n"/>
       <c r="G383" s="3" t="inlineStr">
         <is>
           <t>Human behaviour</t>

</xml_diff>